<commit_message>
archivo SNAPSHOT creado para que sea una misma señal visual e impresa en el exporter
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated_wr_66_pf2.49.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated_wr_66_pf2.49.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\k_99_\Desktop\corridas_exitosas\SPEEDX1_BASELINE\wr_66_pf2.49\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\k_99_\Desktop\codding\OpeningRangeSetup\EddiewareOpeningRangeSetup\EddiewareOpeningRangeSetup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615AFD5D-DCE4-43BD-9801-9DF493F0D994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121239F7-4D22-4A59-89D5-3D6D24FA9990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>

</xml_diff>